<commit_message>
fix: supervision score neutral 5/10 when data absent from CV
When data_missing=True (CV did not include supervision information),
candidates were unfairly penalised with 2/10. Changed to neutral 5/10
since absence of data in CV is not confirmation of zero supervision.
Score of 2/10 is now reserved for confirmed-zero cases only.
Regenerated composite_evaluations.csv with corrected scores.
</commit_message>
<xml_diff>
--- a/data/analysis/composite_evaluations.xlsx
+++ b/data/analysis/composite_evaluations.xlsx
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>86</v>
+        <v>89</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -506,7 +506,7 @@
         <v>25</v>
       </c>
       <c r="F2" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G2" t="n">
         <v>8</v>
@@ -533,7 +533,7 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -547,7 +547,7 @@
         <v>25</v>
       </c>
       <c r="F3" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G3" t="n">
         <v>2</v>
@@ -574,7 +574,7 @@
         </is>
       </c>
       <c r="B4" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -588,7 +588,7 @@
         <v>25</v>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G4" t="n">
         <v>2</v>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B5" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -629,7 +629,7 @@
         <v>25</v>
       </c>
       <c r="F5" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G5" t="n">
         <v>2</v>
@@ -656,7 +656,7 @@
         </is>
       </c>
       <c r="B6" t="n">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -670,7 +670,7 @@
         <v>25</v>
       </c>
       <c r="F6" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G6" t="n">
         <v>2</v>
@@ -697,7 +697,7 @@
         </is>
       </c>
       <c r="B7" t="n">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -711,7 +711,7 @@
         <v>22</v>
       </c>
       <c r="F7" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G7" t="n">
         <v>8</v>
@@ -738,7 +738,7 @@
         </is>
       </c>
       <c r="B8" t="n">
-        <v>80.7</v>
+        <v>83.7</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -752,7 +752,7 @@
         <v>25</v>
       </c>
       <c r="F8" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G8" t="n">
         <v>2</v>
@@ -779,11 +779,11 @@
         </is>
       </c>
       <c r="B9" t="n">
-        <v>79.2</v>
+        <v>82.2</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Tier 2: Strong Candidate</t>
+          <t>Tier 1: Exceptional Fit</t>
         </is>
       </c>
       <c r="D9" t="n">
@@ -793,7 +793,7 @@
         <v>25</v>
       </c>
       <c r="F9" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G9" t="n">
         <v>2</v>
@@ -820,11 +820,11 @@
         </is>
       </c>
       <c r="B10" t="n">
-        <v>78.5</v>
+        <v>81.5</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Tier 2: Strong Candidate</t>
+          <t>Tier 1: Exceptional Fit</t>
         </is>
       </c>
       <c r="D10" t="n">
@@ -834,7 +834,7 @@
         <v>25</v>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G10" t="n">
         <v>2</v>
@@ -861,11 +861,11 @@
         </is>
       </c>
       <c r="B11" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Tier 2: Strong Candidate</t>
+          <t>Tier 1: Exceptional Fit</t>
         </is>
       </c>
       <c r="D11" t="n">
@@ -875,7 +875,7 @@
         <v>22</v>
       </c>
       <c r="F11" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G11" t="n">
         <v>2</v>
@@ -902,11 +902,11 @@
         </is>
       </c>
       <c r="B12" t="n">
-        <v>77</v>
+        <v>80</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Tier 2: Strong Candidate</t>
+          <t>Tier 1: Exceptional Fit</t>
         </is>
       </c>
       <c r="D12" t="n">
@@ -916,7 +916,7 @@
         <v>25</v>
       </c>
       <c r="F12" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G12" t="n">
         <v>2</v>
@@ -943,7 +943,7 @@
         </is>
       </c>
       <c r="B13" t="n">
-        <v>76.7</v>
+        <v>79.7</v>
       </c>
       <c r="C13" t="inlineStr">
         <is>
@@ -957,7 +957,7 @@
         <v>25</v>
       </c>
       <c r="F13" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G13" t="n">
         <v>2</v>
@@ -984,7 +984,7 @@
         </is>
       </c>
       <c r="B14" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C14" t="inlineStr">
         <is>
@@ -998,7 +998,7 @@
         <v>16</v>
       </c>
       <c r="F14" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G14" t="n">
         <v>2</v>
@@ -1025,7 +1025,7 @@
         </is>
       </c>
       <c r="B15" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C15" t="inlineStr">
         <is>
@@ -1039,7 +1039,7 @@
         <v>16</v>
       </c>
       <c r="F15" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G15" t="n">
         <v>2</v>
@@ -1066,7 +1066,7 @@
         </is>
       </c>
       <c r="B16" t="n">
-        <v>75</v>
+        <v>78</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -1080,7 +1080,7 @@
         <v>16</v>
       </c>
       <c r="F16" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G16" t="n">
         <v>2</v>
@@ -1107,7 +1107,7 @@
         </is>
       </c>
       <c r="B17" t="n">
-        <v>74.5</v>
+        <v>77.5</v>
       </c>
       <c r="C17" t="inlineStr">
         <is>
@@ -1121,7 +1121,7 @@
         <v>22</v>
       </c>
       <c r="F17" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G17" t="n">
         <v>2</v>
@@ -1148,7 +1148,7 @@
         </is>
       </c>
       <c r="B18" t="n">
-        <v>74</v>
+        <v>77</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1162,7 +1162,7 @@
         <v>25</v>
       </c>
       <c r="F18" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G18" t="n">
         <v>2</v>
@@ -1189,7 +1189,7 @@
         </is>
       </c>
       <c r="B19" t="n">
-        <v>73.5</v>
+        <v>76.5</v>
       </c>
       <c r="C19" t="inlineStr">
         <is>
@@ -1203,7 +1203,7 @@
         <v>22</v>
       </c>
       <c r="F19" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G19" t="n">
         <v>2</v>
@@ -1230,7 +1230,7 @@
         </is>
       </c>
       <c r="B20" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="C20" t="inlineStr">
         <is>
@@ -1244,7 +1244,7 @@
         <v>16</v>
       </c>
       <c r="F20" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G20" t="n">
         <v>2</v>
@@ -1271,7 +1271,7 @@
         </is>
       </c>
       <c r="B21" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C21" t="inlineStr">
         <is>
@@ -1285,7 +1285,7 @@
         <v>22</v>
       </c>
       <c r="F21" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G21" t="n">
         <v>2</v>
@@ -1312,7 +1312,7 @@
         </is>
       </c>
       <c r="B22" t="n">
-        <v>71</v>
+        <v>74</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1326,7 +1326,7 @@
         <v>22</v>
       </c>
       <c r="F22" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G22" t="n">
         <v>2</v>
@@ -1353,7 +1353,7 @@
         </is>
       </c>
       <c r="B23" t="n">
-        <v>69</v>
+        <v>72</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -1367,7 +1367,7 @@
         <v>16</v>
       </c>
       <c r="F23" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G23" t="n">
         <v>2</v>
@@ -1394,7 +1394,7 @@
         </is>
       </c>
       <c r="B24" t="n">
-        <v>68.5</v>
+        <v>71.5</v>
       </c>
       <c r="C24" t="inlineStr">
         <is>
@@ -1408,7 +1408,7 @@
         <v>16</v>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G24" t="n">
         <v>2</v>
@@ -1435,7 +1435,7 @@
         </is>
       </c>
       <c r="B25" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
       <c r="C25" t="inlineStr">
         <is>
@@ -1449,7 +1449,7 @@
         <v>16</v>
       </c>
       <c r="F25" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G25" t="n">
         <v>2</v>
@@ -1476,7 +1476,7 @@
         </is>
       </c>
       <c r="B26" t="n">
-        <v>67.59999999999999</v>
+        <v>70.59999999999999</v>
       </c>
       <c r="C26" t="inlineStr">
         <is>
@@ -1490,7 +1490,7 @@
         <v>25</v>
       </c>
       <c r="F26" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G26" t="n">
         <v>2</v>
@@ -1517,7 +1517,7 @@
         </is>
       </c>
       <c r="B27" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C27" t="inlineStr">
         <is>
@@ -1531,7 +1531,7 @@
         <v>22</v>
       </c>
       <c r="F27" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G27" t="n">
         <v>2</v>
@@ -1558,7 +1558,7 @@
         </is>
       </c>
       <c r="B28" t="n">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="C28" t="inlineStr">
         <is>
@@ -1572,7 +1572,7 @@
         <v>16</v>
       </c>
       <c r="F28" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G28" t="n">
         <v>2</v>
@@ -1599,7 +1599,7 @@
         </is>
       </c>
       <c r="B29" t="n">
-        <v>66.8</v>
+        <v>69.8</v>
       </c>
       <c r="C29" t="inlineStr">
         <is>
@@ -1613,7 +1613,7 @@
         <v>16</v>
       </c>
       <c r="F29" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G29" t="n">
         <v>2</v>
@@ -1640,7 +1640,7 @@
         </is>
       </c>
       <c r="B30" t="n">
-        <v>66.40000000000001</v>
+        <v>69.40000000000001</v>
       </c>
       <c r="C30" t="inlineStr">
         <is>
@@ -1654,7 +1654,7 @@
         <v>22</v>
       </c>
       <c r="F30" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G30" t="n">
         <v>2</v>
@@ -1681,7 +1681,7 @@
         </is>
       </c>
       <c r="B31" t="n">
-        <v>65</v>
+        <v>68</v>
       </c>
       <c r="C31" t="inlineStr">
         <is>
@@ -1695,7 +1695,7 @@
         <v>16</v>
       </c>
       <c r="F31" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G31" t="n">
         <v>2</v>
@@ -1722,11 +1722,11 @@
         </is>
       </c>
       <c r="B32" t="n">
-        <v>64</v>
+        <v>67</v>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Tier 3: Moderate Candidate</t>
+          <t>Tier 2: Strong Candidate</t>
         </is>
       </c>
       <c r="D32" t="n">
@@ -1736,7 +1736,7 @@
         <v>16</v>
       </c>
       <c r="F32" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G32" t="n">
         <v>2</v>
@@ -1763,11 +1763,11 @@
         </is>
       </c>
       <c r="B33" t="n">
-        <v>63.5</v>
+        <v>66.5</v>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Tier 3: Moderate Candidate</t>
+          <t>Tier 2: Strong Candidate</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -1777,7 +1777,7 @@
         <v>16</v>
       </c>
       <c r="F33" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G33" t="n">
         <v>2</v>
@@ -1804,11 +1804,11 @@
         </is>
       </c>
       <c r="B34" t="n">
-        <v>63</v>
+        <v>66</v>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Tier 3: Moderate Candidate</t>
+          <t>Tier 2: Strong Candidate</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -1818,7 +1818,7 @@
         <v>16</v>
       </c>
       <c r="F34" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G34" t="n">
         <v>2</v>
@@ -1845,11 +1845,11 @@
         </is>
       </c>
       <c r="B35" t="n">
-        <v>62</v>
+        <v>65</v>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Tier 3: Moderate Candidate</t>
+          <t>Tier 2: Strong Candidate</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -1859,7 +1859,7 @@
         <v>16</v>
       </c>
       <c r="F35" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G35" t="n">
         <v>2</v>
@@ -1886,7 +1886,7 @@
         </is>
       </c>
       <c r="B36" t="n">
-        <v>61.5</v>
+        <v>64.5</v>
       </c>
       <c r="C36" t="inlineStr">
         <is>
@@ -1900,7 +1900,7 @@
         <v>16</v>
       </c>
       <c r="F36" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G36" t="n">
         <v>2</v>
@@ -1927,7 +1927,7 @@
         </is>
       </c>
       <c r="B37" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C37" t="inlineStr">
         <is>
@@ -1941,7 +1941,7 @@
         <v>16</v>
       </c>
       <c r="F37" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G37" t="n">
         <v>2</v>
@@ -1968,7 +1968,7 @@
         </is>
       </c>
       <c r="B38" t="n">
-        <v>54.5</v>
+        <v>57.5</v>
       </c>
       <c r="C38" t="inlineStr">
         <is>
@@ -1982,7 +1982,7 @@
         <v>10</v>
       </c>
       <c r="F38" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G38" t="n">
         <v>2</v>
@@ -2009,11 +2009,11 @@
         </is>
       </c>
       <c r="B39" t="n">
-        <v>48.5</v>
+        <v>51.5</v>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Tier 4: Needs Clarification / Weak</t>
+          <t>Tier 3: Moderate Candidate</t>
         </is>
       </c>
       <c r="D39" t="n">
@@ -2023,7 +2023,7 @@
         <v>5</v>
       </c>
       <c r="F39" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G39" t="n">
         <v>2</v>
@@ -2050,7 +2050,7 @@
         </is>
       </c>
       <c r="B40" t="n">
-        <v>45.5</v>
+        <v>48.5</v>
       </c>
       <c r="C40" t="inlineStr">
         <is>
@@ -2064,7 +2064,7 @@
         <v>10</v>
       </c>
       <c r="F40" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G40" t="n">
         <v>2</v>
@@ -2091,7 +2091,7 @@
         </is>
       </c>
       <c r="B41" t="n">
-        <v>44.5</v>
+        <v>47.5</v>
       </c>
       <c r="C41" t="inlineStr">
         <is>
@@ -2105,7 +2105,7 @@
         <v>5</v>
       </c>
       <c r="F41" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G41" t="n">
         <v>2</v>
@@ -2132,7 +2132,7 @@
         </is>
       </c>
       <c r="B42" t="n">
-        <v>44.5</v>
+        <v>47.5</v>
       </c>
       <c r="C42" t="inlineStr">
         <is>
@@ -2146,7 +2146,7 @@
         <v>5</v>
       </c>
       <c r="F42" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G42" t="n">
         <v>2</v>
@@ -2173,7 +2173,7 @@
         </is>
       </c>
       <c r="B43" t="n">
-        <v>41.5</v>
+        <v>44.5</v>
       </c>
       <c r="C43" t="inlineStr">
         <is>
@@ -2187,7 +2187,7 @@
         <v>5</v>
       </c>
       <c r="F43" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G43" t="n">
         <v>2</v>
@@ -2214,7 +2214,7 @@
         </is>
       </c>
       <c r="B44" t="n">
-        <v>32.5</v>
+        <v>35.5</v>
       </c>
       <c r="C44" t="inlineStr">
         <is>
@@ -2228,7 +2228,7 @@
         <v>5</v>
       </c>
       <c r="F44" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G44" t="n">
         <v>2</v>

</xml_diff>